<commit_message>
Refine descriptions and display names in ConceptMap
Updated descriptions and display names for elements in the ConceptMap. 4af5fad9c1a18cd8f14f2a0ab3597e084a64bda1
</commit_message>
<xml_diff>
--- a/traitement-erreur/ig/CdaIIToIdentifierConceptMap.xlsx
+++ b/traitement-erreur/ig/CdaIIToIdentifierConceptMap.xlsx
@@ -8,12 +8,13 @@
   <sheets>
     <sheet name="Metadata" r:id="rId3" sheetId="1"/>
     <sheet name="Mapping Table 0" r:id="rId4" sheetId="2"/>
+    <sheet name="Mapping Table 1" r:id="rId5" sheetId="3"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="54">
   <si>
     <t>Property</t>
   </si>
@@ -24,7 +25,7 @@
     <t>URL</t>
   </si>
   <si>
-    <t>https://interop.esante.gouv.fr/ig/fhir/mappingcdafhir/ConceptMap/DataTypes/CdaIIToIdentifier</t>
+    <t>https://interop.esante.gouv.fr/ig/fhir/mappingcdafhir/ConceptMap/CdaIIToIdentifierConceptMap</t>
   </si>
   <si>
     <t>Version</t>
@@ -60,7 +61,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-22T12:56:04+00:00</t>
+    <t>2026-07-22T13:03:41+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -84,7 +85,7 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Correspondances entre les éléments du datatype CDA II et les éléments FHIR Identifier</t>
+    <t>Correspondances entre les éléments du datatype CDA II et les éléments FHIR Identifier et Reference.</t>
   </si>
   <si>
     <t>Purpose</t>
@@ -117,34 +118,64 @@
     <t>II.extension</t>
   </si>
   <si>
+    <t>Extension</t>
+  </si>
+  <si>
     <t>equivalent</t>
   </si>
   <si>
     <t>Identifier.value</t>
   </si>
   <si>
+    <t>The value that is unique</t>
+  </si>
+  <si>
     <t>II.root</t>
   </si>
   <si>
+    <t>Root</t>
+  </si>
+  <si>
     <t>related-to</t>
   </si>
   <si>
     <t>Identifier.system</t>
   </si>
   <si>
+    <t>The namespace for the identifier value</t>
+  </si>
+  <si>
     <t>II.assigningAuthorityName</t>
   </si>
   <si>
-    <t>Identifier.assigner.display</t>
+    <t>Assigning Authority Name</t>
+  </si>
+  <si>
+    <t>Identifier.assigner</t>
+  </si>
+  <si>
+    <t>Organization that issued id (may be just text)</t>
   </si>
   <si>
     <t>II.displayable</t>
   </si>
   <si>
+    <t>Displayable</t>
+  </si>
+  <si>
     <t>Identifier.extension</t>
   </si>
   <si>
-    <t>Identifier.extension(displayable)</t>
+    <t>Additional content defined by implementations</t>
+  </si>
+  <si>
+    <t>http://hl7.org/fhir/StructureDefinition/Reference|4.0.1</t>
+  </si>
+  <si>
+    <t>Reference.display</t>
+  </si>
+  <si>
+    <t>Text alternative for the resource</t>
   </si>
 </sst>
 </file>
@@ -442,84 +473,145 @@
         <v>33</v>
       </c>
       <c r="B3" t="s" s="2">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C3" t="s" s="2">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D3" t="s" s="2">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E3" t="s" s="2">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="2">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B4" t="s" s="2">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C4" t="s" s="2">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="D4" t="s" s="2">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E4" t="s" s="2">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="2">
+        <v>38</v>
+      </c>
+      <c r="B5" t="s" s="2">
+        <v>39</v>
+      </c>
+      <c r="C5" t="s" s="2">
+        <v>40</v>
+      </c>
+      <c r="D5" t="s" s="2">
         <v>36</v>
       </c>
-      <c r="B5" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="C5" t="s" s="2">
+      <c r="E5" t="s" s="2">
         <v>37</v>
-      </c>
-      <c r="D5" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="E5" t="s" s="2">
-        <v>35</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="2">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B6" t="s" s="2">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="C6" t="s" s="2">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="D6" t="s" s="2">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="E6" t="s" s="2">
-        <v>40</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="2">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="B7" t="s" s="2">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="C7" t="s" s="2">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="D7" t="s" s="2">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="E7" t="s" s="2">
+        <v>50</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="1">
+        <v>26</v>
+      </c>
+      <c r="B1" t="s" s="1">
+        <v>27</v>
+      </c>
+      <c r="C1" t="s" s="1">
+        <v>28</v>
+      </c>
+      <c r="D1" t="s" s="1">
+        <v>29</v>
+      </c>
+      <c r="E1" t="s" s="1">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="2">
+        <v>30</v>
+      </c>
+      <c r="B2" t="s" s="2">
+        <v>31</v>
+      </c>
+      <c r="C2" t="s" s="2">
+        <v>31</v>
+      </c>
+      <c r="D2" t="s" s="2">
+        <v>51</v>
+      </c>
+      <c r="E2" t="s" s="2">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="2">
         <v>43</v>
+      </c>
+      <c r="B3" t="s" s="2">
+        <v>44</v>
+      </c>
+      <c r="C3" t="s" s="2">
+        <v>40</v>
+      </c>
+      <c r="D3" t="s" s="2">
+        <v>52</v>
+      </c>
+      <c r="E3" t="s" s="2">
+        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>